<commit_message>
feat: implementa painel de requisicoes de estoque e fluxo no kanban
</commit_message>
<xml_diff>
--- a/data/tecnicos.xlsx
+++ b/data/tecnicos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://maquinascomprint-my.sharepoint.com/personal/ricardo_almeida_comprint_com_br/Documents/PROJETOS/OUTROS/Programação/chatbot-whatsapp-estoque/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="242" documentId="11_EC77243F16397D4AA023F67958631868A0065613" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0782C49C-AA16-4AE3-B9D0-DA2A7CEDDEC8}"/>
+  <xr:revisionPtr revIDLastSave="263" documentId="11_EC77243F16397D4AA023F67958631868A0065613" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{292FB270-DA9E-445B-B8EB-8BEB53B612B9}"/>
   <bookViews>
-    <workbookView xWindow="-25710" yWindow="880" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tecnicos" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="93">
   <si>
     <t>NOME</t>
   </si>
@@ -309,6 +309,9 @@
   </si>
   <si>
     <t>SKILLS</t>
+  </si>
+  <si>
+    <t>MALA</t>
   </si>
 </sst>
 </file>
@@ -725,17 +728,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E726"/>
-  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:F726"/>
+  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="16.75" customWidth="1"/>
-    <col min="2" max="2" width="19.625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="36.375" customWidth="1"/>
-    <col min="4" max="4" width="19.875" customWidth="1"/>
-    <col min="5" max="5" width="49.375" customWidth="1"/>
+    <col min="2" max="2" width="19.58203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="36.33203125" customWidth="1"/>
+    <col min="4" max="4" width="19.83203125" customWidth="1"/>
+    <col min="5" max="5" width="49.33203125" customWidth="1"/>
+    <col min="6" max="6" width="8.6640625" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -751,8 +755,11 @@
       <c r="E1" t="s">
         <v>91</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F1" s="6" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -760,7 +767,7 @@
         <v>5511980651840</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -768,7 +775,7 @@
         <v>5511974039496</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>25</v>
       </c>
@@ -782,7 +789,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>26</v>
       </c>
@@ -796,7 +803,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -812,8 +819,11 @@
       <c r="E6" t="s">
         <v>79</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F6" s="6">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>5</v>
       </c>
@@ -829,8 +839,11 @@
       <c r="E7" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F7" s="6">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>6</v>
       </c>
@@ -846,8 +859,11 @@
       <c r="E8" t="s">
         <v>79</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F8" s="6">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>7</v>
       </c>
@@ -864,7 +880,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>8</v>
       </c>
@@ -881,7 +897,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>9</v>
       </c>
@@ -897,8 +913,11 @@
       <c r="E11" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F11" s="6">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>10</v>
       </c>
@@ -914,8 +933,11 @@
       <c r="E12" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F12" s="6">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>11</v>
       </c>
@@ -931,8 +953,11 @@
       <c r="E13" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F13" s="6">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>12</v>
       </c>
@@ -948,8 +973,11 @@
       <c r="E14" t="s">
         <v>79</v>
       </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F14" s="6">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>13</v>
       </c>
@@ -965,8 +993,11 @@
       <c r="E15" t="s">
         <v>84</v>
       </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F15" s="6">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>14</v>
       </c>
@@ -974,7 +1005,7 @@
         <v>55133713365</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>15</v>
       </c>
@@ -991,7 +1022,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>16</v>
       </c>
@@ -1007,8 +1038,11 @@
       <c r="E18" t="s">
         <v>79</v>
       </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F18" s="6">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>17</v>
       </c>
@@ -1024,8 +1058,11 @@
       <c r="E19" t="s">
         <v>85</v>
       </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F19" s="6">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>18</v>
       </c>
@@ -1039,7 +1076,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>19</v>
       </c>
@@ -1050,7 +1087,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>20</v>
       </c>
@@ -1066,8 +1103,11 @@
       <c r="E22" t="s">
         <v>79</v>
       </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F22" s="6">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>21</v>
       </c>
@@ -1083,8 +1123,11 @@
       <c r="E23" t="s">
         <v>86</v>
       </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F23" s="6">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>22</v>
       </c>
@@ -1100,8 +1143,11 @@
       <c r="E24" t="s">
         <v>79</v>
       </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F24" s="6">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>28</v>
       </c>
@@ -1117,8 +1163,11 @@
       <c r="E25" t="s">
         <v>87</v>
       </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F25" s="6">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>23</v>
       </c>
@@ -1132,7 +1181,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>24</v>
       </c>
@@ -1145,8 +1194,11 @@
       <c r="D27" t="s">
         <v>70</v>
       </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F27" s="6">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>27</v>
       </c>
@@ -1162,8 +1214,11 @@
       <c r="E28" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F28" s="6">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>29</v>
       </c>
@@ -1179,8 +1234,11 @@
       <c r="E29" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F29" s="6">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>30</v>
       </c>
@@ -1196,8 +1254,11 @@
       <c r="E30" t="s">
         <v>89</v>
       </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F30" s="6">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>31</v>
       </c>
@@ -1213,8 +1274,11 @@
       <c r="E31" t="s">
         <v>90</v>
       </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F31" s="6">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>32</v>
       </c>
@@ -1231,7 +1295,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>33</v>
       </c>
@@ -1248,7 +1312,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>60</v>
       </c>
@@ -1262,7 +1326,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>65</v>
       </c>
@@ -1279,7 +1343,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>67</v>
       </c>
@@ -1293,7 +1357,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>75</v>
       </c>
@@ -1308,7 +1372,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>76</v>
       </c>
@@ -1323,2068 +1387,2068 @@
         <v>90</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B39" s="2"/>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B40" s="2"/>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B41" s="2"/>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B42" s="2"/>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B43" s="2"/>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B44" s="2"/>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B45" s="2"/>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B46" s="2"/>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B47" s="2"/>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B48" s="2"/>
     </row>
-    <row r="49" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="49" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B49" s="2"/>
     </row>
-    <row r="50" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="50" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B50" s="2"/>
     </row>
-    <row r="51" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="51" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B51" s="2"/>
     </row>
-    <row r="52" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="52" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B52" s="2"/>
     </row>
-    <row r="53" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="53" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B53" s="2"/>
     </row>
-    <row r="54" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="54" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B54" s="2"/>
     </row>
-    <row r="55" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="55" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B55" s="2"/>
     </row>
-    <row r="56" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="56" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B56" s="2"/>
     </row>
-    <row r="57" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="57" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B57" s="2"/>
     </row>
-    <row r="58" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="58" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B58" s="2"/>
     </row>
-    <row r="59" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="59" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B59" s="2"/>
     </row>
-    <row r="60" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="60" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B60" s="2"/>
     </row>
-    <row r="61" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="61" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B61" s="2"/>
     </row>
-    <row r="62" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="62" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B62" s="2"/>
     </row>
-    <row r="63" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="63" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B63" s="2"/>
     </row>
-    <row r="64" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="64" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B64" s="2"/>
     </row>
-    <row r="65" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="65" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B65" s="2"/>
     </row>
-    <row r="66" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="66" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B66" s="2"/>
     </row>
-    <row r="67" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="67" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B67" s="2"/>
     </row>
-    <row r="68" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="68" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B68" s="2"/>
     </row>
-    <row r="69" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="69" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B69" s="2"/>
     </row>
-    <row r="70" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="70" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B70" s="2"/>
     </row>
-    <row r="71" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="71" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B71" s="2"/>
     </row>
-    <row r="72" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="72" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B72" s="2"/>
     </row>
-    <row r="73" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="73" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B73" s="2"/>
     </row>
-    <row r="74" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="74" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B74" s="2"/>
     </row>
-    <row r="75" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="75" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B75" s="2"/>
     </row>
-    <row r="76" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="76" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B76" s="2"/>
     </row>
-    <row r="77" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="77" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B77" s="2"/>
     </row>
-    <row r="78" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="78" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B78" s="2"/>
     </row>
-    <row r="79" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="79" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B79" s="2"/>
     </row>
-    <row r="80" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="80" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B80" s="2"/>
     </row>
-    <row r="81" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="81" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B81" s="2"/>
     </row>
-    <row r="82" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="82" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B82" s="2"/>
     </row>
-    <row r="83" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="83" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B83" s="2"/>
     </row>
-    <row r="84" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="84" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B84" s="2"/>
     </row>
-    <row r="85" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="85" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B85" s="2"/>
     </row>
-    <row r="86" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="86" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B86" s="2"/>
     </row>
-    <row r="87" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="87" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B87" s="2"/>
     </row>
-    <row r="88" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="88" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B88" s="2"/>
     </row>
-    <row r="89" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="89" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B89" s="2"/>
     </row>
-    <row r="90" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="90" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B90" s="2"/>
     </row>
-    <row r="91" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="91" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B91" s="2"/>
     </row>
-    <row r="92" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="92" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B92" s="2"/>
     </row>
-    <row r="93" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="93" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B93" s="2"/>
     </row>
-    <row r="94" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="94" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B94" s="2"/>
     </row>
-    <row r="95" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="95" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B95" s="2"/>
     </row>
-    <row r="96" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="96" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B96" s="2"/>
     </row>
-    <row r="97" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="97" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B97" s="2"/>
     </row>
-    <row r="98" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="98" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B98" s="2"/>
     </row>
-    <row r="99" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="99" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B99" s="2"/>
     </row>
-    <row r="100" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="100" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B100" s="2"/>
     </row>
-    <row r="101" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="101" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B101" s="2"/>
     </row>
-    <row r="102" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="102" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B102" s="2"/>
     </row>
-    <row r="103" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="103" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B103" s="2"/>
     </row>
-    <row r="104" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="104" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B104" s="2"/>
     </row>
-    <row r="105" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="105" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B105" s="2"/>
     </row>
-    <row r="106" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="106" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B106" s="2"/>
     </row>
-    <row r="107" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="107" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B107" s="2"/>
     </row>
-    <row r="108" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="108" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B108" s="2"/>
     </row>
-    <row r="109" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="109" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B109" s="2"/>
     </row>
-    <row r="110" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="110" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B110" s="2"/>
     </row>
-    <row r="111" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="111" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B111" s="2"/>
     </row>
-    <row r="112" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="112" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B112" s="2"/>
     </row>
-    <row r="113" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="113" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B113" s="2"/>
     </row>
-    <row r="114" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="114" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B114" s="2"/>
     </row>
-    <row r="115" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="115" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B115" s="2"/>
     </row>
-    <row r="116" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="116" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B116" s="2"/>
     </row>
-    <row r="117" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="117" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B117" s="2"/>
     </row>
-    <row r="118" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="118" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B118" s="2"/>
     </row>
-    <row r="119" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="119" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B119" s="2"/>
     </row>
-    <row r="120" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="120" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B120" s="2"/>
     </row>
-    <row r="121" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="121" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B121" s="2"/>
     </row>
-    <row r="122" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="122" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B122" s="2"/>
     </row>
-    <row r="123" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="123" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B123" s="2"/>
     </row>
-    <row r="124" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="124" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B124" s="2"/>
     </row>
-    <row r="125" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="125" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B125" s="2"/>
     </row>
-    <row r="126" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="126" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B126" s="2"/>
     </row>
-    <row r="127" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="127" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B127" s="2"/>
     </row>
-    <row r="128" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="128" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B128" s="2"/>
     </row>
-    <row r="129" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="129" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B129" s="2"/>
     </row>
-    <row r="130" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="130" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B130" s="2"/>
     </row>
-    <row r="131" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="131" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B131" s="2"/>
     </row>
-    <row r="132" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="132" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B132" s="2"/>
     </row>
-    <row r="133" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="133" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B133" s="2"/>
     </row>
-    <row r="134" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="134" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B134" s="2"/>
     </row>
-    <row r="135" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="135" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B135" s="2"/>
     </row>
-    <row r="136" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="136" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B136" s="2"/>
     </row>
-    <row r="137" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="137" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B137" s="2"/>
     </row>
-    <row r="138" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="138" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B138" s="2"/>
     </row>
-    <row r="139" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="139" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B139" s="2"/>
     </row>
-    <row r="140" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="140" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B140" s="2"/>
     </row>
-    <row r="141" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="141" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B141" s="2"/>
     </row>
-    <row r="142" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="142" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B142" s="2"/>
     </row>
-    <row r="143" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="143" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B143" s="2"/>
     </row>
-    <row r="144" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="144" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B144" s="2"/>
     </row>
-    <row r="145" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="145" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B145" s="2"/>
     </row>
-    <row r="146" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="146" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B146" s="2"/>
     </row>
-    <row r="147" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="147" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B147" s="2"/>
     </row>
-    <row r="148" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="148" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B148" s="2"/>
     </row>
-    <row r="149" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="149" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B149" s="2"/>
     </row>
-    <row r="150" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="150" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B150" s="2"/>
     </row>
-    <row r="151" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="151" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B151" s="2"/>
     </row>
-    <row r="152" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="152" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B152" s="2"/>
     </row>
-    <row r="153" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="153" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B153" s="2"/>
     </row>
-    <row r="154" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="154" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B154" s="2"/>
     </row>
-    <row r="155" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="155" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B155" s="2"/>
     </row>
-    <row r="156" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="156" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B156" s="2"/>
     </row>
-    <row r="157" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="157" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B157" s="2"/>
     </row>
-    <row r="158" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="158" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B158" s="2"/>
     </row>
-    <row r="159" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="159" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B159" s="2"/>
     </row>
-    <row r="160" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="160" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B160" s="2"/>
     </row>
-    <row r="161" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="161" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B161" s="2"/>
     </row>
-    <row r="162" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="162" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B162" s="2"/>
     </row>
-    <row r="163" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="163" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B163" s="2"/>
     </row>
-    <row r="164" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="164" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B164" s="2"/>
     </row>
-    <row r="165" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="165" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B165" s="2"/>
     </row>
-    <row r="166" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="166" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B166" s="2"/>
     </row>
-    <row r="167" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="167" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B167" s="2"/>
     </row>
-    <row r="168" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="168" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B168" s="2"/>
     </row>
-    <row r="169" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="169" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B169" s="2"/>
     </row>
-    <row r="170" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="170" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B170" s="2"/>
     </row>
-    <row r="171" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="171" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B171" s="2"/>
     </row>
-    <row r="172" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="172" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B172" s="2"/>
     </row>
-    <row r="173" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="173" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B173" s="2"/>
     </row>
-    <row r="174" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="174" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B174" s="2"/>
     </row>
-    <row r="175" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="175" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B175" s="2"/>
     </row>
-    <row r="176" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="176" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B176" s="2"/>
     </row>
-    <row r="177" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="177" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B177" s="2"/>
     </row>
-    <row r="178" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="178" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B178" s="2"/>
     </row>
-    <row r="179" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="179" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B179" s="2"/>
     </row>
-    <row r="180" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="180" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B180" s="2"/>
     </row>
-    <row r="181" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="181" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B181" s="2"/>
     </row>
-    <row r="182" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="182" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B182" s="2"/>
     </row>
-    <row r="183" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="183" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B183" s="2"/>
     </row>
-    <row r="184" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="184" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B184" s="2"/>
     </row>
-    <row r="185" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="185" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B185" s="2"/>
     </row>
-    <row r="186" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="186" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B186" s="2"/>
     </row>
-    <row r="187" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="187" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B187" s="2"/>
     </row>
-    <row r="188" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="188" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B188" s="2"/>
     </row>
-    <row r="189" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="189" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B189" s="2"/>
     </row>
-    <row r="190" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="190" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B190" s="2"/>
     </row>
-    <row r="191" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="191" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B191" s="2"/>
     </row>
-    <row r="192" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="192" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B192" s="2"/>
     </row>
-    <row r="193" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="193" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B193" s="2"/>
     </row>
-    <row r="194" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="194" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B194" s="2"/>
     </row>
-    <row r="195" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="195" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B195" s="2"/>
     </row>
-    <row r="196" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="196" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B196" s="2"/>
     </row>
-    <row r="197" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="197" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B197" s="2"/>
     </row>
-    <row r="198" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="198" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B198" s="2"/>
     </row>
-    <row r="199" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="199" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B199" s="2"/>
     </row>
-    <row r="200" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="200" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B200" s="2"/>
     </row>
-    <row r="201" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="201" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B201" s="2"/>
     </row>
-    <row r="202" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="202" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B202" s="2"/>
     </row>
-    <row r="203" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="203" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B203" s="2"/>
     </row>
-    <row r="204" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="204" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B204" s="2"/>
     </row>
-    <row r="205" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="205" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B205" s="2"/>
     </row>
-    <row r="206" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="206" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B206" s="2"/>
     </row>
-    <row r="207" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="207" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B207" s="2"/>
     </row>
-    <row r="208" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="208" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B208" s="2"/>
     </row>
-    <row r="209" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="209" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B209" s="2"/>
     </row>
-    <row r="210" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="210" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B210" s="2"/>
     </row>
-    <row r="211" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="211" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B211" s="2"/>
     </row>
-    <row r="212" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="212" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B212" s="2"/>
     </row>
-    <row r="213" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="213" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B213" s="2"/>
     </row>
-    <row r="214" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="214" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B214" s="2"/>
     </row>
-    <row r="215" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="215" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B215" s="2"/>
     </row>
-    <row r="216" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="216" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B216" s="2"/>
     </row>
-    <row r="217" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="217" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B217" s="2"/>
     </row>
-    <row r="218" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="218" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B218" s="2"/>
     </row>
-    <row r="219" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="219" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B219" s="2"/>
     </row>
-    <row r="220" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="220" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B220" s="2"/>
     </row>
-    <row r="221" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="221" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B221" s="2"/>
     </row>
-    <row r="222" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="222" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B222" s="2"/>
     </row>
-    <row r="223" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="223" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B223" s="2"/>
     </row>
-    <row r="224" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="224" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B224" s="2"/>
     </row>
-    <row r="225" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="225" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B225" s="2"/>
     </row>
-    <row r="226" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="226" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B226" s="2"/>
     </row>
-    <row r="227" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="227" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B227" s="2"/>
     </row>
-    <row r="228" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="228" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B228" s="2"/>
     </row>
-    <row r="229" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="229" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B229" s="2"/>
     </row>
-    <row r="230" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="230" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B230" s="2"/>
     </row>
-    <row r="231" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="231" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B231" s="2"/>
     </row>
-    <row r="232" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="232" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B232" s="2"/>
     </row>
-    <row r="233" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="233" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B233" s="2"/>
     </row>
-    <row r="234" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="234" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B234" s="2"/>
     </row>
-    <row r="235" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="235" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B235" s="2"/>
     </row>
-    <row r="236" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="236" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B236" s="2"/>
     </row>
-    <row r="237" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="237" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B237" s="2"/>
     </row>
-    <row r="238" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="238" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B238" s="2"/>
     </row>
-    <row r="239" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="239" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B239" s="2"/>
     </row>
-    <row r="240" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="240" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B240" s="2"/>
     </row>
-    <row r="241" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="241" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B241" s="2"/>
     </row>
-    <row r="242" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="242" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B242" s="2"/>
     </row>
-    <row r="243" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="243" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B243" s="2"/>
     </row>
-    <row r="244" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="244" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B244" s="2"/>
     </row>
-    <row r="245" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="245" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B245" s="2"/>
     </row>
-    <row r="246" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="246" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B246" s="2"/>
     </row>
-    <row r="247" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="247" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B247" s="2"/>
     </row>
-    <row r="248" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="248" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B248" s="2"/>
     </row>
-    <row r="249" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="249" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B249" s="2"/>
     </row>
-    <row r="250" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="250" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B250" s="2"/>
     </row>
-    <row r="251" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="251" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B251" s="2"/>
     </row>
-    <row r="252" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="252" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B252" s="2"/>
     </row>
-    <row r="253" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="253" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B253" s="2"/>
     </row>
-    <row r="254" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="254" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B254" s="2"/>
     </row>
-    <row r="255" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="255" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B255" s="2"/>
     </row>
-    <row r="256" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="256" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B256" s="2"/>
     </row>
-    <row r="257" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="257" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B257" s="2"/>
     </row>
-    <row r="258" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="258" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B258" s="2"/>
     </row>
-    <row r="259" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="259" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B259" s="2"/>
     </row>
-    <row r="260" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="260" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B260" s="2"/>
     </row>
-    <row r="261" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="261" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B261" s="2"/>
     </row>
-    <row r="262" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="262" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B262" s="2"/>
     </row>
-    <row r="263" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="263" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B263" s="2"/>
     </row>
-    <row r="264" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="264" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B264" s="2"/>
     </row>
-    <row r="265" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="265" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B265" s="2"/>
     </row>
-    <row r="266" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="266" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B266" s="2"/>
     </row>
-    <row r="267" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="267" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B267" s="2"/>
     </row>
-    <row r="268" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="268" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B268" s="2"/>
     </row>
-    <row r="269" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="269" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B269" s="2"/>
     </row>
-    <row r="270" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="270" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B270" s="2"/>
     </row>
-    <row r="271" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="271" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B271" s="2"/>
     </row>
-    <row r="272" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="272" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B272" s="2"/>
     </row>
-    <row r="273" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="273" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B273" s="2"/>
     </row>
-    <row r="274" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="274" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B274" s="2"/>
     </row>
-    <row r="275" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="275" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B275" s="2"/>
     </row>
-    <row r="276" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="276" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B276" s="2"/>
     </row>
-    <row r="277" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="277" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B277" s="2"/>
     </row>
-    <row r="278" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="278" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B278" s="2"/>
     </row>
-    <row r="279" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="279" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B279" s="2"/>
     </row>
-    <row r="280" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="280" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B280" s="2"/>
     </row>
-    <row r="281" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="281" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B281" s="2"/>
     </row>
-    <row r="282" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="282" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B282" s="2"/>
     </row>
-    <row r="283" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="283" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B283" s="2"/>
     </row>
-    <row r="284" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="284" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B284" s="2"/>
     </row>
-    <row r="285" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="285" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B285" s="2"/>
     </row>
-    <row r="286" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="286" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B286" s="2"/>
     </row>
-    <row r="287" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="287" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B287" s="2"/>
     </row>
-    <row r="288" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="288" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B288" s="2"/>
     </row>
-    <row r="289" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="289" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B289" s="2"/>
     </row>
-    <row r="290" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="290" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B290" s="2"/>
     </row>
-    <row r="291" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="291" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B291" s="2"/>
     </row>
-    <row r="292" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="292" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B292" s="2"/>
     </row>
-    <row r="293" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="293" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B293" s="2"/>
     </row>
-    <row r="294" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="294" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B294" s="2"/>
     </row>
-    <row r="295" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="295" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B295" s="2"/>
     </row>
-    <row r="296" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="296" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B296" s="2"/>
     </row>
-    <row r="297" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="297" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B297" s="2"/>
     </row>
-    <row r="298" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="298" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B298" s="2"/>
     </row>
-    <row r="299" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="299" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B299" s="2"/>
     </row>
-    <row r="300" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="300" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B300" s="2"/>
     </row>
-    <row r="301" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="301" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B301" s="2"/>
     </row>
-    <row r="302" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="302" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B302" s="2"/>
     </row>
-    <row r="303" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="303" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B303" s="2"/>
     </row>
-    <row r="304" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="304" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B304" s="2"/>
     </row>
-    <row r="305" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="305" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B305" s="2"/>
     </row>
-    <row r="306" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="306" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B306" s="2"/>
     </row>
-    <row r="307" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="307" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B307" s="2"/>
     </row>
-    <row r="308" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="308" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B308" s="2"/>
     </row>
-    <row r="309" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="309" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B309" s="2"/>
     </row>
-    <row r="310" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="310" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B310" s="2"/>
     </row>
-    <row r="311" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="311" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B311" s="2"/>
     </row>
-    <row r="312" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="312" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B312" s="2"/>
     </row>
-    <row r="313" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="313" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B313" s="2"/>
     </row>
-    <row r="314" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="314" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B314" s="2"/>
     </row>
-    <row r="315" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="315" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B315" s="2"/>
     </row>
-    <row r="316" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="316" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B316" s="2"/>
     </row>
-    <row r="317" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="317" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B317" s="2"/>
     </row>
-    <row r="318" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="318" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B318" s="2"/>
     </row>
-    <row r="319" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="319" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B319" s="2"/>
     </row>
-    <row r="320" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="320" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B320" s="2"/>
     </row>
-    <row r="321" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="321" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B321" s="2"/>
     </row>
-    <row r="322" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="322" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B322" s="2"/>
     </row>
-    <row r="323" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="323" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B323" s="2"/>
     </row>
-    <row r="324" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="324" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B324" s="2"/>
     </row>
-    <row r="325" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="325" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B325" s="2"/>
     </row>
-    <row r="326" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="326" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B326" s="2"/>
     </row>
-    <row r="327" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="327" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B327" s="2"/>
     </row>
-    <row r="328" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="328" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B328" s="2"/>
     </row>
-    <row r="329" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="329" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B329" s="2"/>
     </row>
-    <row r="330" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="330" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B330" s="2"/>
     </row>
-    <row r="331" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="331" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B331" s="2"/>
     </row>
-    <row r="332" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="332" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B332" s="2"/>
     </row>
-    <row r="333" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="333" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B333" s="2"/>
     </row>
-    <row r="334" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="334" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B334" s="2"/>
     </row>
-    <row r="335" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="335" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B335" s="2"/>
     </row>
-    <row r="336" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="336" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B336" s="2"/>
     </row>
-    <row r="337" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="337" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B337" s="2"/>
     </row>
-    <row r="338" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="338" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B338" s="2"/>
     </row>
-    <row r="339" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="339" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B339" s="2"/>
     </row>
-    <row r="340" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="340" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B340" s="2"/>
     </row>
-    <row r="341" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="341" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B341" s="2"/>
     </row>
-    <row r="342" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="342" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B342" s="2"/>
     </row>
-    <row r="343" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="343" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B343" s="2"/>
     </row>
-    <row r="344" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="344" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B344" s="2"/>
     </row>
-    <row r="345" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="345" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B345" s="2"/>
     </row>
-    <row r="346" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="346" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B346" s="2"/>
     </row>
-    <row r="347" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="347" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B347" s="2"/>
     </row>
-    <row r="348" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="348" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B348" s="2"/>
     </row>
-    <row r="349" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="349" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B349" s="2"/>
     </row>
-    <row r="350" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="350" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B350" s="2"/>
     </row>
-    <row r="351" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="351" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B351" s="2"/>
     </row>
-    <row r="352" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="352" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B352" s="2"/>
     </row>
-    <row r="353" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="353" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B353" s="2"/>
     </row>
-    <row r="354" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="354" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B354" s="2"/>
     </row>
-    <row r="355" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="355" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B355" s="2"/>
     </row>
-    <row r="356" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="356" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B356" s="2"/>
     </row>
-    <row r="357" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="357" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B357" s="2"/>
     </row>
-    <row r="358" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="358" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B358" s="2"/>
     </row>
-    <row r="359" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="359" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B359" s="2"/>
     </row>
-    <row r="360" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="360" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B360" s="2"/>
     </row>
-    <row r="361" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="361" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B361" s="2"/>
     </row>
-    <row r="362" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="362" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B362" s="2"/>
     </row>
-    <row r="363" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="363" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B363" s="2"/>
     </row>
-    <row r="364" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="364" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B364" s="2"/>
     </row>
-    <row r="365" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="365" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B365" s="2"/>
     </row>
-    <row r="366" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="366" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B366" s="2"/>
     </row>
-    <row r="367" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="367" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B367" s="2"/>
     </row>
-    <row r="368" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="368" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B368" s="2"/>
     </row>
-    <row r="369" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="369" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B369" s="2"/>
     </row>
-    <row r="370" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="370" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B370" s="2"/>
     </row>
-    <row r="371" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="371" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B371" s="2"/>
     </row>
-    <row r="372" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="372" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B372" s="2"/>
     </row>
-    <row r="373" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="373" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B373" s="2"/>
     </row>
-    <row r="374" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="374" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B374" s="2"/>
     </row>
-    <row r="375" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="375" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B375" s="2"/>
     </row>
-    <row r="376" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="376" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B376" s="2"/>
     </row>
-    <row r="377" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="377" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B377" s="2"/>
     </row>
-    <row r="378" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="378" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B378" s="2"/>
     </row>
-    <row r="379" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="379" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B379" s="2"/>
     </row>
-    <row r="380" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="380" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B380" s="2"/>
     </row>
-    <row r="381" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="381" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B381" s="2"/>
     </row>
-    <row r="382" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="382" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B382" s="2"/>
     </row>
-    <row r="383" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="383" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B383" s="2"/>
     </row>
-    <row r="384" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="384" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B384" s="2"/>
     </row>
-    <row r="385" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="385" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B385" s="2"/>
     </row>
-    <row r="386" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="386" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B386" s="2"/>
     </row>
-    <row r="387" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="387" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B387" s="2"/>
     </row>
-    <row r="388" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="388" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B388" s="2"/>
     </row>
-    <row r="389" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="389" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B389" s="2"/>
     </row>
-    <row r="390" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="390" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B390" s="2"/>
     </row>
-    <row r="391" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="391" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B391" s="2"/>
     </row>
-    <row r="392" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="392" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B392" s="2"/>
     </row>
-    <row r="393" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="393" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B393" s="2"/>
     </row>
-    <row r="394" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="394" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B394" s="2"/>
     </row>
-    <row r="395" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="395" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B395" s="2"/>
     </row>
-    <row r="396" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="396" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B396" s="2"/>
     </row>
-    <row r="397" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="397" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B397" s="2"/>
     </row>
-    <row r="398" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="398" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B398" s="2"/>
     </row>
-    <row r="399" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="399" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B399" s="2"/>
     </row>
-    <row r="400" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="400" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B400" s="2"/>
     </row>
-    <row r="401" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="401" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B401" s="2"/>
     </row>
-    <row r="402" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="402" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B402" s="2"/>
     </row>
-    <row r="403" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="403" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B403" s="2"/>
     </row>
-    <row r="404" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="404" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B404" s="2"/>
     </row>
-    <row r="405" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="405" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B405" s="2"/>
     </row>
-    <row r="406" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="406" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B406" s="2"/>
     </row>
-    <row r="407" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="407" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B407" s="2"/>
     </row>
-    <row r="408" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="408" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B408" s="2"/>
     </row>
-    <row r="409" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="409" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B409" s="2"/>
     </row>
-    <row r="410" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="410" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B410" s="2"/>
     </row>
-    <row r="411" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="411" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B411" s="2"/>
     </row>
-    <row r="412" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="412" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B412" s="2"/>
     </row>
-    <row r="413" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="413" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B413" s="2"/>
     </row>
-    <row r="414" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="414" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B414" s="2"/>
     </row>
-    <row r="415" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="415" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B415" s="2"/>
     </row>
-    <row r="416" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="416" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B416" s="2"/>
     </row>
-    <row r="417" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="417" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B417" s="2"/>
     </row>
-    <row r="418" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="418" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B418" s="2"/>
     </row>
-    <row r="419" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="419" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B419" s="2"/>
     </row>
-    <row r="420" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="420" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B420" s="2"/>
     </row>
-    <row r="421" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="421" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B421" s="2"/>
     </row>
-    <row r="422" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="422" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B422" s="2"/>
     </row>
-    <row r="423" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="423" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B423" s="2"/>
     </row>
-    <row r="424" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="424" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B424" s="2"/>
     </row>
-    <row r="425" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="425" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B425" s="2"/>
     </row>
-    <row r="426" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="426" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B426" s="2"/>
     </row>
-    <row r="427" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="427" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B427" s="2"/>
     </row>
-    <row r="428" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="428" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B428" s="2"/>
     </row>
-    <row r="429" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="429" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B429" s="2"/>
     </row>
-    <row r="430" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="430" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B430" s="2"/>
     </row>
-    <row r="431" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="431" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B431" s="2"/>
     </row>
-    <row r="432" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="432" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B432" s="2"/>
     </row>
-    <row r="433" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="433" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B433" s="2"/>
     </row>
-    <row r="434" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="434" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B434" s="2"/>
     </row>
-    <row r="435" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="435" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B435" s="2"/>
     </row>
-    <row r="436" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="436" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B436" s="2"/>
     </row>
-    <row r="437" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="437" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B437" s="2"/>
     </row>
-    <row r="438" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="438" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B438" s="2"/>
     </row>
-    <row r="439" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="439" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B439" s="2"/>
     </row>
-    <row r="440" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="440" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B440" s="2"/>
     </row>
-    <row r="441" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="441" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B441" s="2"/>
     </row>
-    <row r="442" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="442" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B442" s="2"/>
     </row>
-    <row r="443" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="443" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B443" s="2"/>
     </row>
-    <row r="444" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="444" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B444" s="2"/>
     </row>
-    <row r="445" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="445" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B445" s="2"/>
     </row>
-    <row r="446" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="446" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B446" s="2"/>
     </row>
-    <row r="447" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="447" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B447" s="2"/>
     </row>
-    <row r="448" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="448" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B448" s="2"/>
     </row>
-    <row r="449" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="449" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B449" s="2"/>
     </row>
-    <row r="450" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="450" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B450" s="2"/>
     </row>
-    <row r="451" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="451" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B451" s="2"/>
     </row>
-    <row r="452" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="452" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B452" s="2"/>
     </row>
-    <row r="453" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="453" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B453" s="2"/>
     </row>
-    <row r="454" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="454" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B454" s="2"/>
     </row>
-    <row r="455" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="455" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B455" s="2"/>
     </row>
-    <row r="456" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="456" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B456" s="2"/>
     </row>
-    <row r="457" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="457" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B457" s="2"/>
     </row>
-    <row r="458" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="458" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B458" s="2"/>
     </row>
-    <row r="459" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="459" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B459" s="2"/>
     </row>
-    <row r="460" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="460" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B460" s="2"/>
     </row>
-    <row r="461" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="461" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B461" s="2"/>
     </row>
-    <row r="462" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="462" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B462" s="2"/>
     </row>
-    <row r="463" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="463" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B463" s="2"/>
     </row>
-    <row r="464" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="464" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B464" s="2"/>
     </row>
-    <row r="465" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="465" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B465" s="2"/>
     </row>
-    <row r="466" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="466" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B466" s="2"/>
     </row>
-    <row r="467" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="467" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B467" s="2"/>
     </row>
-    <row r="468" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="468" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B468" s="2"/>
     </row>
-    <row r="469" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="469" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B469" s="2"/>
     </row>
-    <row r="470" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="470" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B470" s="2"/>
     </row>
-    <row r="471" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="471" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B471" s="2"/>
     </row>
-    <row r="472" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="472" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B472" s="2"/>
     </row>
-    <row r="473" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="473" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B473" s="2"/>
     </row>
-    <row r="474" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="474" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B474" s="2"/>
     </row>
-    <row r="475" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="475" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B475" s="2"/>
     </row>
-    <row r="476" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="476" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B476" s="2"/>
     </row>
-    <row r="477" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="477" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B477" s="2"/>
     </row>
-    <row r="478" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="478" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B478" s="2"/>
     </row>
-    <row r="479" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="479" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B479" s="2"/>
     </row>
-    <row r="480" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="480" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B480" s="2"/>
     </row>
-    <row r="481" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="481" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B481" s="2"/>
     </row>
-    <row r="482" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="482" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B482" s="2"/>
     </row>
-    <row r="483" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="483" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B483" s="2"/>
     </row>
-    <row r="484" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="484" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B484" s="2"/>
     </row>
-    <row r="485" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="485" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B485" s="2"/>
     </row>
-    <row r="486" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="486" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B486" s="2"/>
     </row>
-    <row r="487" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="487" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B487" s="2"/>
     </row>
-    <row r="488" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="488" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B488" s="2"/>
     </row>
-    <row r="489" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="489" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B489" s="2"/>
     </row>
-    <row r="490" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="490" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B490" s="2"/>
     </row>
-    <row r="491" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="491" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B491" s="2"/>
     </row>
-    <row r="492" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="492" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B492" s="2"/>
     </row>
-    <row r="493" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="493" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B493" s="2"/>
     </row>
-    <row r="494" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="494" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B494" s="2"/>
     </row>
-    <row r="495" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="495" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B495" s="2"/>
     </row>
-    <row r="496" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="496" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B496" s="2"/>
     </row>
-    <row r="497" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="497" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B497" s="2"/>
     </row>
-    <row r="498" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="498" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B498" s="2"/>
     </row>
-    <row r="499" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="499" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B499" s="2"/>
     </row>
-    <row r="500" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="500" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B500" s="2"/>
     </row>
-    <row r="501" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="501" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B501" s="2"/>
     </row>
-    <row r="502" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="502" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B502" s="2"/>
     </row>
-    <row r="503" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="503" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B503" s="2"/>
     </row>
-    <row r="504" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="504" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B504" s="2"/>
     </row>
-    <row r="505" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="505" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B505" s="2"/>
     </row>
-    <row r="506" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="506" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B506" s="2"/>
     </row>
-    <row r="507" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="507" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B507" s="2"/>
     </row>
-    <row r="508" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="508" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B508" s="2"/>
     </row>
-    <row r="509" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="509" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B509" s="2"/>
     </row>
-    <row r="510" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="510" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B510" s="2"/>
     </row>
-    <row r="511" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="511" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B511" s="2"/>
     </row>
-    <row r="512" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="512" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B512" s="2"/>
     </row>
-    <row r="513" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="513" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B513" s="2"/>
     </row>
-    <row r="514" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="514" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B514" s="2"/>
     </row>
-    <row r="515" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="515" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B515" s="2"/>
     </row>
-    <row r="516" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="516" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B516" s="2"/>
     </row>
-    <row r="517" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="517" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B517" s="2"/>
     </row>
-    <row r="518" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="518" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B518" s="2"/>
     </row>
-    <row r="519" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="519" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B519" s="2"/>
     </row>
-    <row r="520" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="520" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B520" s="2"/>
     </row>
-    <row r="521" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="521" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B521" s="2"/>
     </row>
-    <row r="522" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="522" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B522" s="2"/>
     </row>
-    <row r="523" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="523" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B523" s="2"/>
     </row>
-    <row r="524" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="524" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B524" s="2"/>
     </row>
-    <row r="525" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="525" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B525" s="2"/>
     </row>
-    <row r="526" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="526" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B526" s="2"/>
     </row>
-    <row r="527" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="527" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B527" s="2"/>
     </row>
-    <row r="528" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="528" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B528" s="2"/>
     </row>
-    <row r="529" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="529" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B529" s="2"/>
     </row>
-    <row r="530" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="530" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B530" s="2"/>
     </row>
-    <row r="531" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="531" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B531" s="2"/>
     </row>
-    <row r="532" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="532" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B532" s="2"/>
     </row>
-    <row r="533" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="533" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B533" s="2"/>
     </row>
-    <row r="534" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="534" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B534" s="2"/>
     </row>
-    <row r="535" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="535" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B535" s="2"/>
     </row>
-    <row r="536" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="536" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B536" s="2"/>
     </row>
-    <row r="537" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="537" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B537" s="2"/>
     </row>
-    <row r="538" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="538" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B538" s="2"/>
     </row>
-    <row r="539" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="539" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B539" s="2"/>
     </row>
-    <row r="540" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="540" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B540" s="2"/>
     </row>
-    <row r="541" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="541" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B541" s="2"/>
     </row>
-    <row r="542" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="542" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B542" s="2"/>
     </row>
-    <row r="543" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="543" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B543" s="2"/>
     </row>
-    <row r="544" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="544" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B544" s="2"/>
     </row>
-    <row r="545" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="545" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B545" s="2"/>
     </row>
-    <row r="546" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="546" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B546" s="2"/>
     </row>
-    <row r="547" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="547" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B547" s="2"/>
     </row>
-    <row r="548" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="548" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B548" s="2"/>
     </row>
-    <row r="549" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="549" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B549" s="2"/>
     </row>
-    <row r="550" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="550" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B550" s="2"/>
     </row>
-    <row r="551" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="551" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B551" s="2"/>
     </row>
-    <row r="552" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="552" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B552" s="2"/>
     </row>
-    <row r="553" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="553" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B553" s="2"/>
     </row>
-    <row r="554" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="554" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B554" s="2"/>
     </row>
-    <row r="555" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="555" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B555" s="2"/>
     </row>
-    <row r="556" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="556" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B556" s="2"/>
     </row>
-    <row r="557" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="557" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B557" s="2"/>
     </row>
-    <row r="558" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="558" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B558" s="2"/>
     </row>
-    <row r="559" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="559" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B559" s="2"/>
     </row>
-    <row r="560" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="560" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B560" s="2"/>
     </row>
-    <row r="561" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="561" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B561" s="2"/>
     </row>
-    <row r="562" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="562" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B562" s="2"/>
     </row>
-    <row r="563" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="563" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B563" s="2"/>
     </row>
-    <row r="564" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="564" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B564" s="2"/>
     </row>
-    <row r="565" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="565" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B565" s="2"/>
     </row>
-    <row r="566" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="566" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B566" s="2"/>
     </row>
-    <row r="567" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="567" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B567" s="2"/>
     </row>
-    <row r="568" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="568" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B568" s="2"/>
     </row>
-    <row r="569" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="569" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B569" s="2"/>
     </row>
-    <row r="570" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="570" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B570" s="2"/>
     </row>
-    <row r="571" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="571" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B571" s="2"/>
     </row>
-    <row r="572" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="572" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B572" s="2"/>
     </row>
-    <row r="573" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="573" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B573" s="2"/>
     </row>
-    <row r="574" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="574" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B574" s="2"/>
     </row>
-    <row r="575" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="575" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B575" s="2"/>
     </row>
-    <row r="576" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="576" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B576" s="2"/>
     </row>
-    <row r="577" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="577" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B577" s="2"/>
     </row>
-    <row r="578" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="578" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B578" s="2"/>
     </row>
-    <row r="579" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="579" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B579" s="2"/>
     </row>
-    <row r="580" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="580" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B580" s="2"/>
     </row>
-    <row r="581" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="581" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B581" s="2"/>
     </row>
-    <row r="582" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="582" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B582" s="2"/>
     </row>
-    <row r="583" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="583" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B583" s="2"/>
     </row>
-    <row r="584" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="584" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B584" s="2"/>
     </row>
-    <row r="585" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="585" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B585" s="2"/>
     </row>
-    <row r="586" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="586" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B586" s="2"/>
     </row>
-    <row r="587" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="587" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B587" s="2"/>
     </row>
-    <row r="588" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="588" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B588" s="2"/>
     </row>
-    <row r="589" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="589" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B589" s="2"/>
     </row>
-    <row r="590" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="590" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B590" s="2"/>
     </row>
-    <row r="591" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="591" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B591" s="2"/>
     </row>
-    <row r="592" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="592" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B592" s="2"/>
     </row>
-    <row r="593" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="593" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B593" s="2"/>
     </row>
-    <row r="594" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="594" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B594" s="2"/>
     </row>
-    <row r="595" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="595" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B595" s="2"/>
     </row>
-    <row r="596" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="596" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B596" s="2"/>
     </row>
-    <row r="597" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="597" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B597" s="2"/>
     </row>
-    <row r="598" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="598" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B598" s="2"/>
     </row>
-    <row r="599" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="599" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B599" s="2"/>
     </row>
-    <row r="600" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="600" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B600" s="2"/>
     </row>
-    <row r="601" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="601" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B601" s="2"/>
     </row>
-    <row r="602" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="602" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B602" s="2"/>
     </row>
-    <row r="603" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="603" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B603" s="2"/>
     </row>
-    <row r="604" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="604" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B604" s="2"/>
     </row>
-    <row r="605" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="605" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B605" s="2"/>
     </row>
-    <row r="606" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="606" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B606" s="2"/>
     </row>
-    <row r="607" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="607" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B607" s="2"/>
     </row>
-    <row r="608" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="608" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B608" s="2"/>
     </row>
-    <row r="609" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="609" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B609" s="2"/>
     </row>
-    <row r="610" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="610" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B610" s="2"/>
     </row>
-    <row r="611" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="611" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B611" s="2"/>
     </row>
-    <row r="612" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="612" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B612" s="2"/>
     </row>
-    <row r="613" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="613" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B613" s="2"/>
     </row>
-    <row r="614" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="614" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B614" s="2"/>
     </row>
-    <row r="615" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="615" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B615" s="2"/>
     </row>
-    <row r="616" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="616" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B616" s="2"/>
     </row>
-    <row r="617" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="617" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B617" s="2"/>
     </row>
-    <row r="618" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="618" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B618" s="2"/>
     </row>
-    <row r="619" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="619" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B619" s="2"/>
     </row>
-    <row r="620" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="620" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B620" s="2"/>
     </row>
-    <row r="621" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="621" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B621" s="2"/>
     </row>
-    <row r="622" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="622" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B622" s="2"/>
     </row>
-    <row r="623" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="623" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B623" s="2"/>
     </row>
-    <row r="624" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="624" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B624" s="2"/>
     </row>
-    <row r="625" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="625" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B625" s="2"/>
     </row>
-    <row r="626" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="626" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B626" s="2"/>
     </row>
-    <row r="627" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="627" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B627" s="2"/>
     </row>
-    <row r="628" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="628" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B628" s="2"/>
     </row>
-    <row r="629" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="629" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B629" s="2"/>
     </row>
-    <row r="630" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="630" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B630" s="2"/>
     </row>
-    <row r="631" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="631" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B631" s="2"/>
     </row>
-    <row r="632" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="632" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B632" s="2"/>
     </row>
-    <row r="633" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="633" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B633" s="2"/>
     </row>
-    <row r="634" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="634" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B634" s="2"/>
     </row>
-    <row r="635" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="635" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B635" s="2"/>
     </row>
-    <row r="636" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="636" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B636" s="2"/>
     </row>
-    <row r="637" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="637" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B637" s="2"/>
     </row>
-    <row r="638" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="638" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B638" s="2"/>
     </row>
-    <row r="639" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="639" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B639" s="2"/>
     </row>
-    <row r="640" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="640" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B640" s="2"/>
     </row>
-    <row r="641" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="641" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B641" s="2"/>
     </row>
-    <row r="642" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="642" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B642" s="2"/>
     </row>
-    <row r="643" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="643" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B643" s="2"/>
     </row>
-    <row r="644" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="644" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B644" s="2"/>
     </row>
-    <row r="645" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="645" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B645" s="2"/>
     </row>
-    <row r="646" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="646" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B646" s="2"/>
     </row>
-    <row r="647" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="647" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B647" s="2"/>
     </row>
-    <row r="648" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="648" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B648" s="2"/>
     </row>
-    <row r="649" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="649" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B649" s="2"/>
     </row>
-    <row r="650" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="650" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B650" s="2"/>
     </row>
-    <row r="651" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="651" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B651" s="2"/>
     </row>
-    <row r="652" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="652" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B652" s="2"/>
     </row>
-    <row r="653" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="653" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B653" s="2"/>
     </row>
-    <row r="654" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="654" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B654" s="2"/>
     </row>
-    <row r="655" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="655" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B655" s="2"/>
     </row>
-    <row r="656" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="656" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B656" s="2"/>
     </row>
-    <row r="657" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="657" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B657" s="2"/>
     </row>
-    <row r="658" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="658" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B658" s="2"/>
     </row>
-    <row r="659" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="659" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B659" s="2"/>
     </row>
-    <row r="660" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="660" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B660" s="2"/>
     </row>
-    <row r="661" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="661" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B661" s="2"/>
     </row>
-    <row r="662" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="662" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B662" s="2"/>
     </row>
-    <row r="663" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="663" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B663" s="2"/>
     </row>
-    <row r="664" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="664" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B664" s="2"/>
     </row>
-    <row r="665" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="665" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B665" s="2"/>
     </row>
-    <row r="666" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="666" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B666" s="1"/>
     </row>
-    <row r="667" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="667" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B667" s="1"/>
     </row>
-    <row r="668" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="668" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B668" s="1"/>
     </row>
-    <row r="669" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="669" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B669" s="1"/>
     </row>
-    <row r="670" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="670" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B670" s="1"/>
     </row>
-    <row r="671" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="671" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B671" s="1"/>
     </row>
-    <row r="672" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="672" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B672" s="1"/>
     </row>
-    <row r="673" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="673" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B673" s="1"/>
     </row>
-    <row r="674" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="674" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B674" s="1"/>
     </row>
-    <row r="675" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="675" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B675" s="1"/>
     </row>
-    <row r="676" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="676" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B676" s="1"/>
     </row>
-    <row r="677" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="677" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B677" s="1"/>
     </row>
-    <row r="678" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="678" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B678" s="1"/>
     </row>
-    <row r="679" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="679" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B679" s="1"/>
     </row>
-    <row r="680" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="680" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B680" s="1"/>
     </row>
-    <row r="681" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="681" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B681" s="1"/>
     </row>
-    <row r="682" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="682" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B682" s="1"/>
     </row>
-    <row r="683" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="683" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B683" s="1"/>
     </row>
-    <row r="684" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="684" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B684" s="1"/>
     </row>
-    <row r="685" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="685" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B685" s="1"/>
     </row>
-    <row r="686" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="686" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B686" s="1"/>
     </row>
-    <row r="687" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="687" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B687" s="1"/>
     </row>
-    <row r="688" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="688" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B688" s="1"/>
     </row>
-    <row r="689" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="689" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B689" s="1"/>
     </row>
-    <row r="690" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="690" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B690" s="1"/>
     </row>
-    <row r="691" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="691" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B691" s="1"/>
     </row>
-    <row r="692" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="692" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B692" s="1"/>
     </row>
-    <row r="693" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="693" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B693" s="1"/>
     </row>
-    <row r="694" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="694" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B694" s="1"/>
     </row>
-    <row r="695" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="695" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B695" s="1"/>
     </row>
-    <row r="696" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="696" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B696" s="1"/>
     </row>
-    <row r="697" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="697" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B697" s="1"/>
     </row>
-    <row r="698" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="698" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B698" s="1"/>
     </row>
-    <row r="699" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="699" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B699" s="1"/>
     </row>
-    <row r="700" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="700" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B700" s="1"/>
     </row>
-    <row r="701" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="701" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B701" s="1"/>
     </row>
-    <row r="702" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="702" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B702" s="1"/>
     </row>
-    <row r="703" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="703" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B703" s="1"/>
     </row>
-    <row r="704" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="704" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B704" s="1"/>
     </row>
-    <row r="705" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="705" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B705" s="1"/>
     </row>
-    <row r="706" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="706" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B706" s="1"/>
     </row>
-    <row r="707" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="707" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B707" s="1"/>
     </row>
-    <row r="708" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="708" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B708" s="1"/>
     </row>
-    <row r="709" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="709" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B709" s="1"/>
     </row>
-    <row r="710" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="710" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B710" s="1"/>
     </row>
-    <row r="711" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="711" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B711" s="1"/>
     </row>
-    <row r="712" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="712" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B712" s="1"/>
     </row>
-    <row r="713" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="713" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B713" s="1"/>
     </row>
-    <row r="714" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="714" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B714" s="1"/>
     </row>
-    <row r="715" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="715" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B715" s="1"/>
     </row>
-    <row r="716" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="716" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B716" s="1"/>
     </row>
-    <row r="717" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="717" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B717" s="1"/>
     </row>
-    <row r="718" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="718" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B718" s="1"/>
     </row>
-    <row r="719" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="719" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B719" s="1"/>
     </row>
-    <row r="720" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="720" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B720" s="1"/>
     </row>
-    <row r="721" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="721" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B721" s="1"/>
     </row>
-    <row r="722" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="722" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B722" s="1"/>
     </row>
-    <row r="723" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="723" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B723" s="1"/>
     </row>
-    <row r="724" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="724" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B724" s="1"/>
     </row>
-    <row r="725" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="725" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B725" s="1"/>
     </row>
-    <row r="726" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="726" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B726" s="1"/>
     </row>
   </sheetData>

</xml_diff>